<commit_message>
Update ISMB abstract and author info
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/author_info.xlsx
+++ b/author_info.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="52">
   <si>
     <t xml:space="preserve">Family name</t>
   </si>
@@ -121,6 +121,9 @@
     <t xml:space="preserve">shenrunx@broadinstitute.org</t>
   </si>
   <si>
+    <t xml:space="preserve">0000-0002-8883-5496</t>
+  </si>
+  <si>
     <t xml:space="preserve">Imaging Platform, Broad Institute of Harvard and MIT, Cambridge, Massachusetts, United States</t>
   </si>
   <si>
@@ -133,6 +136,9 @@
     <t xml:space="preserve">steverozen@pm.me</t>
   </si>
   <si>
+    <t xml:space="preserve">0000-0002-4288-0056</t>
+  </si>
+  <si>
     <t xml:space="preserve">Boot</t>
   </si>
   <si>
@@ -158,6 +164,18 @@
   </si>
   <si>
     <t xml:space="preserve">husky0927@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">China</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Molecular Cancer Research Center, School of Medicine, Shenzhen Campus of Sun Yat-Sen University</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sino-French Hoffmann Institute, School of Basic Medical Sciences, Guangzhou Medical University</t>
+  </si>
+  <si>
+    <t xml:space="preserve">United States</t>
   </si>
 </sst>
 </file>
@@ -245,7 +263,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -258,7 +276,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="justify" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -268,6 +286,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -290,37 +312,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -393,25 +415,23 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="137.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="24.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="61.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0"/>
-      <c r="D1" s="0"/>
-    </row>
-    <row r="2" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="2" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -421,10 +441,10 @@
       <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
     </row>
@@ -438,10 +458,10 @@
       <c r="C3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -455,10 +475,10 @@
       <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -472,10 +492,11 @@
       <c r="C5" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="4"/>
+      <c r="E5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>16</v>
       </c>
     </row>
@@ -489,10 +510,11 @@
       <c r="C6" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="5"/>
+      <c r="E6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>25</v>
       </c>
     </row>
@@ -506,14 +528,15 @@
       <c r="C7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="4"/>
+      <c r="E7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="F7" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>30</v>
       </c>
@@ -523,52 +546,194 @@
       <c r="C8" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="D8" s="4"/>
+      <c r="E8" s="1" t="s">
         <v>33</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="D9" s="4"/>
+      <c r="E9" s="1" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>42</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="D16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -578,6 +743,10 @@
     <hyperlink ref="C8" r:id="rId3" display="shenrunx@broadinstitute.org"/>
     <hyperlink ref="C9" r:id="rId4" display="steverozen@pm.me"/>
     <hyperlink ref="C16" r:id="rId5" display="shenli0721@gmail.com"/>
+    <hyperlink ref="C26" r:id="rId6" display="zhengqi2727@gmail.com"/>
+    <hyperlink ref="C28" r:id="rId7" display="Yangying@163.com"/>
+    <hyperlink ref="C29" r:id="rId8" display="shenrunx@broadinstitute.org"/>
+    <hyperlink ref="C30" r:id="rId9" display="steverozen@pm.me"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>